<commit_message>
feat(datasets): generate 25 Frontend Developer questions across all categories
</commit_message>
<xml_diff>
--- a/supabase/question_bank_master.xlsx
+++ b/supabase/question_bank_master.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,7 +464,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Technical</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,17 +474,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Apa perbedaan antara State dan Props dalam React, dan kapan Anda menggunakan masing-masing?</t>
+          <t>Ceritakan tentang pengalaman Anda membangun aplikasi Frontend dan stack teknologi yang paling sering Anda gunakan.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{Penjelasan State,Penjelasan Props,Immutability,Data flow top-down}</t>
+          <t>{Latar belakang pengalaman Frontend,Framework utama (React/Next.js/Vue),State management &amp; Styling kit,Pencapaian proyek utama}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Situation: Anggota tim pemula kebingungan mengelola data komponen. Task: Menjelaskan best practice. Action: Mengedukasi bahwa Props bersifat read-only dari parent dan State adalah mutable lokal. Result: Struktur komponen tim lebih teratur.</t>
+          <t>Situation: Memulai karir 3 tahun sebagai Frontend Engineer. Task: Mengembangkan aplikasi web interaktif skala sedang-besar. Action: Memanfaatkan React, TypeScript, TailwindCSS, dan Zustand untuk arsitektur clean. Result: Berhasil merilis 4 aplikasi web dengan performa tinggi dan kepuasan pengguna 95%.</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -499,27 +499,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Technical</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>easy</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bagaimana Anda mengoptimalkan performa aplikasi React yang mengalami re-render berlebihan?</t>
+          <t>Bagaimana cara Anda tetap up-to-date dengan perkembangan ekosistem Frontend yang berubah sangat cepat?</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{React.memo,useCallback,useMemo,Code splitting/lazy loading,Virtualization}</t>
+          <t>{Membaca dokumentasi resmi &amp; changelog,Mengikuti newsletter/blog seperti React Status &amp; Vercel,Eksperimen side-project,Komunitas lokal/global}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Situation: Halaman dashboard terasa lambat saat scroll data besar. Task: Mengurangi re-render tak perlu. Action: Menggunakan React.memo untuk item list dan useMemo untuk kalkulasi berat. Result: FPS naik dari 30 ke 60 FPS.</t>
+          <t>Situation: Ekosistem Frontend berinovasi sangat cepat seperti Server Actions dan Compiler baru. Task: Menjaga keahlian tetap relevan. Action: Membaca RFC resmi, mencoba fitur baru di side-project akhir pekan, dan mendiskusikan temuan di tech-sharing mingguan tim. Result: Tim dapat mengadopsi optimasi build terbaru lebih cepat.</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -534,30 +534,800 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Apa perbedaan antara State dan Props dalam React, dan kapan Anda menggunakan masing-masing?</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{Penjelasan State (mutable lokal),Penjelasan Props (immutable dari parent),Data flow top-down,Kapan menggunakan masing-masing}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Situation: Anggota tim pemula kebingungan mengelola data komponen. Task: Menjelaskan best practice data flow. Action: Mengedukasi bahwa Props bersifat read-only dari parent dan State adalah mutable lokal. Result: Struktur komponen tim menjadi lebih teratur dan bebas bug re-render.</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Jelaskan bagaimana Event Delegation bekerja pada JavaScript dan mengapa hal ini penting untuk efisiensi DOM?</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{Event Bubbling &amp; Capturing,Single Event Listener pada parent,Penghematan memori,Penanganan elemen dinamis}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Situation: List produk dengan 1000+ item memiliki event listener terpasang pada tiap item, membuat memori melonjak. Task: Memperbaiki efisiensi memori DOM. Action: Menerapkan Event Delegation dengan memasang 1 listener di elemen parent &lt;ul&gt; dan menggunakan e.target. Result: Penggunaan memori DOM berkurang 70%.</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Apa perbedaan utama antara CSS Flexbox dan CSS Grid, serta kapan waktu terbaik menggunakan masing-masing?</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{Flexbox untuk 1 dimensi (row/column),CSS Grid untuk 2 dimensi (row &amp; column),Use case spesifik masing-masing,Alignment &amp; distribution}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Situation: Layout dashboard kompleks bertabrakan di tampilan mobile. Task: Merapikan tata letak komponen. Action: Menggunakan CSS Grid untuk struktur utama dashboard (2D) dan Flexbox untuk aligment navbar &amp; tombol (1D). Result: Tampilan fully responsive di semua ukuran layar.</t>
+        </is>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bagaimana cara kerja useEffect Hook dan bagaimana Anda mencegah timbulnya infinite re-render atau memory leak?</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{Dependency Array (empty, populated, missing),Cleanup function (unsubscribe/abort),Stale closure problem,Strict Mode double-invoke}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Situation: Fitur live notification mengalami memory leak dan request berulang ke API. Task: Memperbaiki lifecycle effect. Action: Mengisi dependency array dengan tepat dan menambahkan cleanup function return () =&gt; socket.disconnect(). Result: Kebocoran memori teratasi dan konsumsi CPU stabil.</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Kapan Anda memilih menggunakan Local State (useState), Context API, atau Global State Manager seperti Zustand/Redux?</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{Local State untuk komponen terisolasi,Context API untuk low-velocity global data (theme/auth),Zustand/Redux untuk high-velocity &amp; complex state,Avoid prop drilling}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Situation: Aplikasi mengalami prop drilling hingga 5 level komponen untuk data keranjang belanja. Task: Memilih state architecture yang scalable. Action: Menggunakan Zustand untuk keranjang belanja agar komponen hanya re-render pada selector yang berubah. Result: Kode bersih dan render terpangkas 50%.</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Bagaimana TypeScript membantu Anda mencegah runtime error di Frontend, dan apa bedanya Type vs Interface?</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{Static type checking,Autocomplete &amp; DX,Interface declaration merging,Type alias union/intersection}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Situation: Sering terjadi TypeError: Cannot read property of undefined saat konsumsi API backend. Task: Mengurangi bug runtime. Action: Mengadopsi TypeScript secara ketat dengan interface kontrak DTO API. Result: Bug runtime di production berkurang hingga 80%.</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda menangani race condition pada API request yang dipanggil berturut-turut saat user mengetik di search bar?</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{Debouncing / Throttling,AbortController (cancelling stale request),Race condition identification,UX loading state}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Situation: Hasil pencarian di UI menampilkan data yang salah jika request lambat selesai belakangan. Task: Menjamin data pencarian selalu sesuai ketikan terakhir. Action: Mengombinasikan Debounce 300ms dengan AbortController.abort() pada request sebelumnya. Result: Hasil pencarian 100% konsisten.</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Jelaskan perbedaan antara Client-Side Rendering (CSR), Server-Side Rendering (SSR), dan Static Site Generation (SSG).</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{CSR (SPA/React),SSR (Next.js server render per request),SSG (Pre-rendered build time),Impact pada SEO &amp; Time to First Byte (TTFB)}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Situation: Landing page produk memiliki skor SEO buruk di Google Search. Task: Meningkatkan keterbacaan bot SEO. Action: Memindahkan landing page dari CSR ke SSG/SSR menggunakan Next.js. Result: Skor Lighthouse SEO naik dari 45 ke 98 dan indexing Google lebih cepat.</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Apa yang dimaksud dengan Mismatch Hydration pada SSR (Next.js/Astro) dan bagaimana cara mendiagnosis serta memperbaikinya?</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{Penyebab: Perbedaan HTML Server vs DOM Client,Server-side vs Client-side evaluation (window/localStorage/Date),SuppressHydrationWarning vs useEffect mounting,Debugging console error}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Situation: Console prod dipenuhi error Hydration failed because initial UI does not match. Task: Menghilangkan error hydration. Action: Memindahkan akses localStorage dan Date.now() ke dalam useEffect setelah komponen dipastikan mounted di client. Result: Error hydration bersih total.</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bagaimana langkah-langkah Anda mengoptimalkan performa aplikasi React yang mengalami re-render berlebihan dan bundle size membengkak?</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{React Profiler analysis,React.memo &amp; useCallback/useMemo,Tree shaking &amp; dynamic import,Bundle analyzer}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Situation: Ukuran JS bundle utama mencapai 4.5 MB. Task: Mengurangi bundle size &amp; TTI. Action: Menganalisis via Bundle Analyzer, mengganti moment.js dengan dayjs, dan menerapkan code-splitting per route. Result: Ukuran bundle turun ke 800 KB dan TTI membaik 60%.</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda meningkatkan nilai Core Web Vitals (LCP, INP, CLS) pada website e-commerce yang memiliki banyak gambar dan skrip pihak ketiga?</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{LCP: Next/Image optimization &amp; fetchpriority,INP: Yielding to main thread (requestIdleCallback/setTimeout),CLS: Reserved dimension ratios (width/height),Third-party script deferring}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Situation: Nilai Core Web Vitals merah di Search Console karena gambar banner besar dan script analytics. Task: Mencapai status Green Vitals. Action: Menggunakan format WebP/AVIF dengan srcset, menset fetchpriority=high untuk hero image, dan defer analytics script. Result: LCP turun dari 4.2s ke 1.8s dan INP &lt; 150ms.</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda mengimplementasikan strategi Lazy Loading dan Dynamic Import untuk rute dan komponen berat?</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{React.lazy &amp; Suspense,Dynamic import import(),Fallback skeleton loader,Intersection Observer untuk image/section}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Situation: Halaman Checkout mendownload modal heavy chart padahal jarang dibuka. Task: Memuat komponen hanya saat dibutuhkan. Action: Membungkus komponen Chart dengan React.lazy() dan Suspense fallback. Result: Initial page load berkurang 350 KB.</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>System Design</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>hard</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Bagaimana Anda merancang arsitektur Micro-Frontend untuk aplikasi web skala besar?</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>{Module Federation,Single-spa,Shared State Management,Routing,CSS Isolation}</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Situation: 5 tim frontend saling bertabrakan saat merilis fitur. Task: Memisah aplikasi menjadi modul independen. Action: Menggunakan Webpack Module Federation dengan shell app. Result: Tim dapat deploy secara independen tanpa bug regresi.</t>
-        </is>
-      </c>
-      <c r="G4" t="b">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda merancang arsitektur Micro-Frontend untuk aplikasi skala besar yang dikerjakan oleh beberapa tim terpisah?</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{Module Federation (Webpack 5 / Vite),Single-spa / Shell app pattern,Shared state &amp; Event Bus,CSS Isolation,Independent Deployment Pipeline}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Situation: 5 tim frontend saling bertabrakan rilis karena monolit web app. Task: Memisah aplikasi menjadi modul independen. Action: Menggunakan Webpack Module Federation dengan shell app dan shared design system. Result: Tim dapat deploy modul secara independen tanpa bug regresi.</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>System Design</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda merancang Design System dan Component Library yang terisolasi, re-usable, dan teruji untuk digunakan di seluruh tim organisasi?</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{Atomic Design Methodology,Storybook for documentation,Tailwind / CSS Variables design tokens,Radix / Headless UI for accessibility,NPM Private Package / Monorepo release}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Situation: Setiap aplikasi internal perusahaan memiliki tampilan tombol dan modal yang konsisten. Task: Mengstandardisasi UI komponen. Action: Membangun Design System berbasis Tailwind &amp; Radix UI di Monorepo dengan Storybook. Result: Kecepatan pengembangan UI baru meningkat 40%.</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>System Design</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda merancang arsitektur web app Offline-First menggunakan Service Workers dan IndexedDB?</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{Service Worker Caching (Stale-While-Revalidate/Cache First),IndexedDB storage via Dexie.js,Background Sync API,Conflict resolution on reconnect}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Situation: Aplikasi inspeksi lapangan sering digunakan di daerah tanpa sinyal internet. Task: Mendukung akses offline penuh. Action: Menerapkan Workbox Service Worker dan IndexedDB untuk menyimpan draf formulir lokal dengan sync otomatis saat online. Result: Pengguna dapat bekerja tanpa hambatan koneksi.</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda mencegah serangan XSS (Cross-Site Scripting) dan CSRF pada aplikasi Web Single Page Application (SPA)?</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{Sanitasi HTML (DOMPurify),Hindari dangerouslySetInnerHTML,Content Security Policy (CSP) headers,SameSite Cookies vs Anti-CSRF Tokens}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Situation: Fitur komentar pengguna rentan disisipi skrip jahat. Task: Mengamankan UI dari XSS. Action: Menggunakan DOMPurify untuk mensanitasi input kaya teks dan memasang strict CSP header pada web server. Result: Aplikasi aman dari eksekusi script injeksi.</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Di mana lokasi terbaik menyimpan Access Token dan Refresh Token di Frontend dari sudut pandang keamanan?</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{HttpOnly SameSite Cookie (Paling aman),In-Memory (JS variable) untuk Access Token,Bahaya localStorage/sessionStorage terhadap XSS,Silent refresh pattern}</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Situation: Token JWT disimpan di localStorage sehingga rentan dibaca oleh script terinjeksi XSS. Task: Mengamankan mekanisme autentikasi. Action: Mengubah simpanan Refresh Token ke HttpOnly SameSite Cookie dan Access Token di in-memory state. Result: Kredensial pengguna terlindungi dari pencurian token.</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mengapa Accessibility (a11y) penting dan bagaimana Anda memastikan komponen web dapat diakses navigasi keyboard dan Screen Reader?</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{Semantic HTML elements,ARIA attributes (aria-label, aria-expanded),Focus management &amp; Focus rings,Screen reader testing (NVDA/VoiceOver)}</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Situation: Modal custom tidak bisa ditutup dengan tombol ESC dan fokus keyboard jebol ke latar belakang. Task: Memperbaiki aksesibilitas modal. Action: Menerapkan Focus Trap dan mendengarkan event keydown ESC serta menambahkan aria-modal=true. Result: Modal lolos pengujian audit WCAG AA.</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman saat Anda berbeda pendapat dengan UI/UX Designer mengenai fungsionalitas komponen yang sulit diimplementasikan.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{Empati terhadap pengguna &amp; desainer,Analisis kepraktisan &amp; trade-off teknis,Kompromi &amp; alternatif prototype,Pengambilan keputusan berbasis data}</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Situation: Desainer membuat efek animasi 3D kompleks di halaman checkout yang berisiko menurunkan performa HP low-end. Task: Mencapai kesepakatan terbaik. Action: Membuat 2 prototype cepat (efek 3D vs CSS micro-animation) dan menunjukkan dampak latency-nya. Result: Tim sepakat memakai micro-animation yang ringan dan estetik.</t>
+        </is>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ceritakan insiden bug kritis yang terjadi di production Frontend dan bagaimana langkah penanganan Anda dari rilis hotfix hingga post-mortem.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>{Triage &amp; isolasi masalah,Rollback vs Hotfix cepat,Komunikasi dengan tim &amp; stakeholder,Post-mortem &amp; penambahan regression test}</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Situation: Tombol bayar tidak bisa diklik pada browser Safari setelah rilis malam. Task: Mengatasi bug kritis secepatnya. Action: Mengidentifikasi polyfill CSS gap pada Safari, merilis hotfix dalam 20 menit, dan menambahkan E2E test Playwright untuk Safari di CI/CD. Result: Kerugian transaksi berhasil diminimalisir.</t>
+        </is>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda meyakinkan Product Manager untuk memberikan alokasi waktu refactoring legacy frontend code yang sudah berantakan?</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{Menerjemahkan tech debt menjadi dampak bisnis (kecepatan rilis/bug rate),Menyajikan data metrics (Lighthouse/Build time),Refactoring bertahap (boy scout rule),Bukan rewrite total}</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Situation: Kode codebase lama membuat waktu pengembangan fitur baru melambat 2 kali lipat. Task: Mendapatkan approval refactoring dari PM. Action: Menyajikan data bahwa 60% waktu sprint habis untuk bug-fixing akibat tech debt dan mengusulkan refactoring bertahap di tiap sprint (20%). Result: PM setuju dan kecepatan rilis meningkat 35%.</t>
+        </is>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman Anda membantu atau mentoring junior developer dalam memahami best practice modern Frontend.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>{Code Review bertahap dengan penjelasan alasan (the why),Pair programming,Dokumentasi &amp; Guideline,Mendukung rasa percaya diri}</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Situation: Junior dev sering mengalami kendala pemahaman async JavaScript dan state management. Task: Membantu meningkatkan keahlian junior dev. Action: Mengadakan sesi pair programming mingguan dan memberikan feedback code review yang konstruktif beserta link referensi. Result: Junior dev mampu menyelesaikan tugas mandiri tanpa blocker.</t>
+        </is>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bagaimana Anda mengelola kualitas kode dan testing ketika dihadapkan pada tenggat waktu rilis fitur yang sangat ketat?</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{Fokus pada Critical Path testing (Unit test core logic &amp; E2E checkout),Pragmatic trade-off (manual QA vs automated test),Linter &amp; Automated formatting (ESLint/Prettier),Dokumentasi sisa debt}</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Situation: Fitur promo baru harus rilis dalam 2 hari untuk campaign marketing. Task: Memastikan fitur rilis tepat waktu tanpa merusak fungsi kritis. Action: Menulis Unit Test khusus untuk kalkulasi diskon dan E2E test untuk alur checkout, sementara komponen UI dites manual. Result: Fitur rilis tepat waktu zero-critical bug.</t>
+        </is>
+      </c>
+      <c r="G26" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(datasets): generate 25 General interview questions across all behavioral & competency categories
</commit_message>
<xml_diff>
--- a/supabase/question_bank_master.xlsx
+++ b/supabase/question_bank_master.xlsx
@@ -1619,7 +1619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1667,30 +1667,870 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ceritakan tentang diri Anda dan latar belakang pengalaman profesional Anda secara singkat.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{Latar belakang profesional,Keahlian &amp; fokus utama,Pencapaian relevan,Alasan antusiasme peranan}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Situation: Membuka sesi wawancara kerja. Task: Memberikan gambaran kualifikasi dalam 2 menit. Action: Menjelaskan 3+ tahun pengalaman di bidang pengembangan software, pencapaian mengoptimalkan performa web 40%, dan minat pada produk inovatif perusahaan ini. Result: Pewawancara mendapatkan gambaran latar belakang yang solid.</t>
+        </is>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mengapa Anda tertarik untuk melamar posisi dan bergabung di perusahaan kami?</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{Pemahaman kultur &amp; produk perusahaan,Relevansi nilai pribadi dengan visi perusahaan,Kontribusi yang ingin diberikan}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Situation: Tertarik melamar karena reputasi inovasi produk perusahaan. Task: Menunjukkan motivasi dan fit kultur. Action: Menjelaskan riset produk terkini perusahaan dan bagaimana keahlian saya dapat mengakselerasi pengembangan fitur tersebut. Result: Membuktikan ketertarikan yang genuine dan persiapan matang.</t>
+        </is>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Apa kekuatan atau keahlian utama yang paling membedakan Anda dengan kandidat lain?</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{Skill spesifik yang relevan,Contoh nyata penerapan kekuatan,Dampak positif pada tim/proyek}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Situation: Menyoroti keunggulan kompetitif. Task: Mengomunikasikan keahlian utama. Action: Menjelaskan kombinasi keahlian teknis pemecahan masalah (problem-solving) dan komunikasi yang efektif antara tim engineering dan bisnis. Result: Pewawancara memahami nilai tambah unik saya.</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Apa kelemahan terbesar Anda dan bagaimana usaha konkret yang Anda lakukan untuk mengatasinya?</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{Kelemahan nyata (bukan perfectionist),Langkah perbaikan konkret,Perkembangan/progres saat ini}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Situation: Dulu sering mengalami kesulitan mengatakan tidak pada tugas tambahan. Task: Mengatasi kelemahan manajemen waktu. Action: Belajar menggunakan framework prioritisasi RICE dan mendiskusikan kapasitas kerja secara terbuka dengan manajer. Result: Produktivitas meningkat tanpa beban berlebih.</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ceritakan pencapaian paling berkesan dalam karir/studi Anda dan bagaimana proses Anda mencapainya.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{Tantangan awal,Langkah strategis,Metrik keberhasilan,Dampak jangka panjang}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Situation: Proyek aplikasi web mengalami kendala keandalan di tengah peluncuran. Task: Memastikan stabilitas sistem. Action: Memimpin migrasi arsitektur ke microservices dan otomatisasi testing dalam waktu 1 bulan. Result: Aplikasi berhasil rilis zero-downtime dan meraih 50,000 pengguna baru.</t>
+        </is>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Di mana Anda melihat diri Anda sendiri dalam 3 hingga 5 tahun ke depan?</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{Tujuan karir realistis,Pengembangan skill jangka panjang,Kontribusi pada pertumbuhan perusahaan}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Situation: Merencanakan jalur karir jangka panjang. Task: Menyelaraskan ambisi dengan arah perusahaan. Action: Berkomitmen memperdalam penguasaan teknologi frontend/fullstack dan bercita-cita tumbuh menjadi Tech Lead yang membimbing tim. Result: Pewawancara melihat komitmen loyalitas dan motivasi berkembang.</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Behavioral</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman Anda ketika dihadapkan pada masalah yang sangat rumit dan bagaimana Anda menyelesaikannya.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{Identifikasi akar masalah (Root Cause),Metode analisis terstruktur,Implementasi solusi,Evaluasi hasil}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Situation: Terjadi bug sporadis di production yang sulit di-reproduce. Task: Mencari dan menangani bug. Action: Mengumpulkan telemetry log, melakukan profiling memori, dan mengisolasi race condition pada komponen state. Result: Bug berhasil diperbaiki permanen dan stabilitas mencapai 99.9%.</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman saat Anda mengalami konflik atau perbedaan pendapat dengan rekan kerja/atasan.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{Mendengarkan aktif (Active listening),Fokus pada tujuan bersama,Diskusi berbasis data/bukti,Kompromi win-win}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Situation: Perbedaan pandangan dengan UI designer terkait kompleksitas animasi fitur. Task: Mencapai kesepakatan terbaik. Action: Mengajak diskusi dengan prototype pembanding serta menyajikan data performa perangkat low-end. Result: Sepakat memilih animasi yang ringan namun tetap estetik.</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ceritakan kegagalan atau kesalahan terbesar yang pernah Anda buat di tempat kerja dan pelajaran apa yang Anda dapatkan.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{Tanggung jawab tanpa menyalahkan orang lain,Tindakan korektif cepat,Pelajaran &amp; mitigasi masa depan}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Situation: Pernah secara tidak sengaja salah deploy skrip database di staging yang merusak draf data testing. Task: Memperbaiki kesalahan dengan jujur. Action: Segera menginformasikan tim, melakukan rollback dari backup, dan memasang guard Script Migration CI/CD. Result: Data pulih dan sistem CI/CD menjadi lebih aman.</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Bagaimana cara Anda mengelola stres dan tetap produktif ketika tenggat waktu sangat mendesak?</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{Manajemen emosi &amp; ketenangan,Breakdown tugas skala kecil,Komunikasi transparansi status,Fokus pada prioritas utama}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Situation: Fitur kritis ditargetkan rilis dalam 2 hari untuk event launching. Task: Menjaga kualitas di bawah tekanan. Action: Membuat urutan tugas prioritas utama (critical path), mengomunikasikan progres tiap 4 jam, dan fokus tanpa distraksi. Result: Fitur rilis tepat waktu tanpa bug penahan.</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Ceritakan tentang diri Anda dan mengapa Anda tertarik dengan posisi ini.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>{Latar belakang singkat,Pencapaian utama,Alasan tertarik pada perusahaan,Relevansi keahlian}</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Situation: Pembuka wawancara kerja. Task: Memberikan impresi awal yang kuat dalam 2 menit. Action: Menjelaskan background 3 tahun di software dev dan passion pada AI products. Result: Pewawancara tertarik mendalami pengalaman proyek AI saya.</t>
-        </is>
-      </c>
-      <c r="G2" t="b">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Berikan contoh situasi di mana Anda harus bekerja sama dengan anggota tim yang memiliki kepribadian/gaya kerja yang berbeda.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{Empati &amp; toleransi gaya kerja,Komunikasi yang jelas,Menyesuaikan pendekatan kolaborasi,Saling melengkapi keahlian}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Situation: Bekerja dengan anggota tim senior yang sangat perfeksionis dan tertutup. Task: Membangun kolaborasi harmonis. Action: Rutin mengajukan pertanyaan terstruktur di sesi kaji kode dan meminta masukan dengan penuh respek. Result: Hubungan kerja menjadi sangat solid dan saling percaya.</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman saat perusahaan/proyek mengalami perubahan arah secara mendadak (pivoting) dan bagaimana Anda beradaptasi.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{Sikap fleksibel &amp; positif,Re-prioritisasi tugas,Mempelajari skill baru secepatnya,Menjaga fokus tim}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Situation: Arah produk berubah dari aplikasi desktop ke aplikasi berbasis web PWA. Task: Beradaptasi dengan teknologi baru. Action: Mengikuti kursus intensif PWA dalam 1 minggu dan merancang ulang arsitektur sistem. Result: Berhasil melakukan peluncuran PWA versi beta dalam 1 bulan.</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ceritakan situasi ketika Anda mengambil inisiatif untuk memperbaiki suatu proses tanpa diminta oleh atasan.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{Inisiatif pribadi (Proactivity),Identifikasi efisiensi proses,Eksekusi mandiri,Dampak peningkatan produktivitas}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Situation: Dokumentasi onboarding dev baru kurang lengkap dan memperlambat tim. Task: Meningkatkan efisiensi onboarding. Action: Secara mandiri mendokumentasikan setup environment dan membuat script setup otomatis. Result: Waktu onboarding dev baru terangkas dari 3 hari menjadi 3 jam.</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Bagaimana cara Anda memprioritaskan tugas saat Anda memiliki beberapa proyek dengan tenggat waktu yang bersamaan?</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{Eisenhower Matrix / RICE framework,Komunikasi tenggat waktu ke stakeholder,Delegasi / Negotiation scope,Fokus eksekusi}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Situation: Mendapat 3 permintaan fitur darurat dari tim marketing dan produk bersamaan. Task: Menentukan prioritas yang tepat. Action: Berdiskusi dengan manajer untuk mengevaluasi dampak bisnis dari masing-masing fitur dan membuat timeline rilis bertahap. Result: Semua proyek selesai tepat waktu sesuai ekspetasi.</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman saat Anda menerima kritik atau umpan balik negatif, dan bagaimana Anda meresponnya.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{Menerima kritik secara profesional (tidak defensif),Evaluasi diri secara objektif,Tindakan perbaikan konkret,Follow-up hasil}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Situation: Menerima masukan dari tim QA bahwa kode saya kurang memiliki penanganan error boundary. Task: Memperbaiki kualitas kode. Action: Mengucapkan terima kasih atas masukkan tersebut dan segera menerapkan Error Boundary pada komponen utama. Result: Kuantitas crash log di Sentry berkurang 80%.</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ceritakan pengalaman saat Anda harus memimpin suatu proyek atau membimbing rekan tim yang sedang kesulitan.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{Empati &amp; mendengar kendala,Memberikan arahan &amp; panduan clear,Memfasilitasi blocker,Merayakan keberhasilan bersama}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Situation: Rekan tim junior kesulitan memahami integrasi sistem autentikasi OAuth. Task: Membantu hingga mandiri. Action: Mengadakan sesi pair programming 1 jam dan menyusun dokumentasi flowchart alur autentikasi. Result: Rekan tim berhasil menyelesaikan modul OAuth dan percaya diri.</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Bagaimana cara Anda menangani klien atau stakeholder yang menuntut hal-hal yang tidak realistis?</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{Mendengarkan kebutuhan inti,Menjelaskan keterbatasan teknis/waktu secara sopan,Menawarkan solusi alternatif realistis,Menjaga ekspektasi}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Situation: Klien meminta perubahan desain total 2 hari sebelum rilis. Task: Mengelola ekspektasi tanpa merusak hubungan. Action: Menjelaskan dampak risiko pada kualitas dan menawarkan rilis bertahap (fitur inti dulu, sisanya di fase 2). Result: Klien menerima dan puas dengan hasil rilis.</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ceritakan keputusan tersulit yang pernah Anda buat di tempat kerja saat informasi yang dimiliki sangat terbatas.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{Analisis risiko &amp; skenario terbaik/terburuk,Menggunakan kalkulasi berbasis intuisi &amp; data ada,Tanggung jawab penuh atas hasil,Evaluasi pasca keputusan}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Situation: Harus memilih library UI baru saat proyek baru mulai tanpa tahu kebutuhan lengkap masa depan. Task: Mengambil keputusan cepat. Action: Mengatur kriteria evaluasi (ukuran bundle, populasi komunitas, keaktifan maintenance) dan memilih Tailwind+Radix. Result: Arsitektur UI tetap relevan dan scalable hingga sekarang.</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Keterampilan baru apa yang Anda pelajari sendiri dalam 6 bulan terakhir dan bagaimana Anda menerapkannya?</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{Inisiatif belajar mandiri,Metode pembelajaran (buku/kursus/proyek),Penerapan praktis pada pekerjaan}</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Situation: Ingin menguasai teknik performa web terkini. Task: Belajar mandiri mengenai Core Web Vitals. Action: Mengikuti dokumentasi web.dev dan mempraktikkannya pada side project. Result: Menerapkan optimasi LCP pada project kantor dan menaikkan score Lighthouse 30 poin.</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Apa arti integritas dan etika kerja bagi Anda, serta bagaimana Anda menerapkannya sehari-hari?</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{Kejujuran &amp; transparansi,Konsistensi komitmen,Menjaga kerahasiaan data perusahaan,Tanggung jawab profesional}</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Situation: Menghadapi situasi di mana ada celah untuk mengambil jalan pintas yang berisiko pada keamanan data. Task: Menjaga integritas. Action: Menolak jalan pintas tersebut dan melaporkan risiko keamanan kepada lead. Result: Keamanan data pengguna tetap terjaga 100%.</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Berikan contoh ketika Anda berusaha melebihi ekspektasi untuk memuaskan kebutuhan pelanggan atau pengguna.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{Mengerti pain point pengguna,Memberikan nilai tambah ekstra,Perhatian terhadap detail UX,Dampak positif umpan balik}</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Situation: Pengguna mengeluhkan kesulitan membaca teks saat mode gelap (dark mode). Task: Memperbaiki kenyamanan pengguna. Action: Mengubah kontras warna sesuai standar WCAG AA dan menambahkan tombol penyesuaian ukuran font. Result: Ulasan positif pengguna meningkat drastis.</t>
+        </is>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bagaimana cara Anda menjelaskan konsep teknis/kompleks kepada rekan kerja non-teknis agar mudah dipahami?</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>{Menggunakan analogi sederhana,Menghindari jargon teknis rumit,Fokus pada manfaat bisnis/pengguna,Menggunakan visual/diagram}</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Situation: Menjelaskan alasan mengapa refactoring database penting kepada tim Marketing. Task: Menyampaikan tanpa jargon. Action: Menggunakan analogi "merapikan gudang toko agar pelayan bisa mengambil barang lebih cepat". Result: Tim Marketing paham dan menyetujui jadwal maintenance.</t>
+        </is>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mengapa Anda memutuskan untuk mencari kesempatan baru atau meninggalkan posisi Anda yang sekarang?</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{Fokus pada pertumbuhan karir &amp; tantangan baru,Apresiasi pada perusahaan lama (tidak menjelekkan),Relevansi tujuan dengan posisi baru}</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Situation: Telah mencapai titik pembelajaran maksimal di posisi lama selama 2.5 tahun. Task: Mencari tempat tumbuh baru. Action: Mencari tantangan baru di perusahaan berteknologi tinggi yang memfasilitasi dampak skala lebih besar. Result: Siap memberikan kontribusi terbaik di posisi ini.</t>
+        </is>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Lingkungan kerja seperti apa yang membuat Anda dapat memberikan performa terbaik Anda?</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>{Kultur kolaboratif &amp; terbuka,Komunikasi transparan,Dukungan inovasi &amp; eksplorasi,Keseimbangan kerja-hidup}</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Situation: Berkembang di lingkungan kerja yang mengutamakan trust dan ownership. Task: Menilai kecocokan budaya. Action: Berkontribusi aktif pada lingkungan yang saling mensupport, mengapresiasi ide baru, dan memiliki feedback loop yang sehat. Result: Produktivitas dan hasil kerja maksimal.</t>
+        </is>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Apakah ada pertanyaan yang ingin Anda ajukan kepada kami mengenai tim, peran, atau budaya perusahaan?</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{Persiapan pertanyaan berbobot,Ketertarikan pada ekspektasi peranan,Antusiasme terhadap pertumbuhan tim}</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Situation: Kesempatan bertanya di akhir sesi wawancara. Task: Menunjukkan ketertarikan mendalam. Action: Menanyakan mengenai indikator sukses 90 hari pertama di posisi ini dan tantangan terbesar yang sedang dihadapi tim saat ini. Result: Memberikan kesan akhir yang sangat profesional dan proaktif.</t>
+        </is>
+      </c>
+      <c r="G26" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>